<commit_message>
Veille des prix : exemple de correspondances sur trois plats
Risotto poulet chorizo, lentilles lardons et ramen : 31 lignes
ingrédient × enseigne pré-remplies dans le carnet Excel, liens à coller.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SZpg93hHD1m9z8kyX4WvDA
</commit_message>
<xml_diff>
--- a/outils/veille-prix/donnees/carnet_produits.xlsx
+++ b/outils/veille-prix/donnees/carnet_produits.xlsx
@@ -424,17 +424,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H34"/>
+  <dimension ref="A1:H32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
     <col width="45" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="9" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -475,536 +475,1062 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>recettes (info)</t>
+          <t>plat (info)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>huile d'olive</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr"/>
-      <c r="C2" t="inlineStr"/>
+          <t>riz arborio</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>leclerc</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>riz pour risotto arborio</t>
+        </is>
+      </c>
       <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
       <c r="G2" t="inlineStr"/>
-      <c r="H2" t="n">
-        <v>8</v>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>risotto poulet chorizo</t>
+        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>riz</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr"/>
-      <c r="C3" t="inlineStr"/>
+          <t>riz arborio</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>amazon</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>riz arborio ou carnaroli</t>
+        </is>
+      </c>
       <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
       <c r="G3" t="inlineStr"/>
-      <c r="H3" t="n">
-        <v>6</v>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>risotto poulet chorizo</t>
+        </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ail</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="inlineStr"/>
+          <t>blancs de poulet</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>leclerc</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>filets de poulet</t>
+        </is>
+      </c>
       <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
       <c r="G4" t="inlineStr"/>
-      <c r="H4" t="n">
-        <v>5</v>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>risotto poulet chorizo</t>
+        </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>épices de base</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr"/>
-      <c r="C5" t="inlineStr"/>
+          <t>blancs de poulet</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>carrefour</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>filets de poulet</t>
+        </is>
+      </c>
       <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
       <c r="G5" t="inlineStr"/>
-      <c r="H5" t="n">
-        <v>5</v>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>risotto poulet chorizo</t>
+        </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>oignons</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr"/>
-      <c r="C6" t="inlineStr"/>
+          <t>chorizo</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>leclerc</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>chorizo doux en bâton</t>
+        </is>
+      </c>
       <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>250</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
       <c r="G6" t="inlineStr"/>
-      <c r="H6" t="n">
-        <v>4</v>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>risotto poulet chorizo</t>
+        </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>sauce soja</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr"/>
-      <c r="C7" t="inlineStr"/>
+          <t>chorizo</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>intermarche</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>chorizo doux en bâton</t>
+        </is>
+      </c>
       <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>250</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
       <c r="G7" t="inlineStr"/>
-      <c r="H7" t="n">
-        <v>3</v>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>risotto poulet chorizo</t>
+        </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>œufs</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr"/>
-      <c r="C8" t="inlineStr"/>
+          <t>bouillon de volaille</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>leclerc</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>bouillon cube volaille</t>
+        </is>
+      </c>
       <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>pièce</t>
+        </is>
+      </c>
       <c r="G8" t="inlineStr"/>
-      <c r="H8" t="n">
-        <v>3</v>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>risotto poulet chorizo</t>
+        </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>blancs de poulet</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr"/>
-      <c r="C9" t="inlineStr"/>
+          <t>vin blanc sec</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>carrefour</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>vin blanc sec de cuisine</t>
+        </is>
+      </c>
       <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>75</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>cl</t>
+        </is>
+      </c>
       <c r="G9" t="inlineStr"/>
-      <c r="H9" t="n">
-        <v>2</v>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>risotto poulet chorizo</t>
+        </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>citrons</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr"/>
-      <c r="C10" t="inlineStr"/>
+          <t>parmesan</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>leclerc</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>parmesan râpé</t>
+        </is>
+      </c>
       <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
       <c r="G10" t="inlineStr"/>
-      <c r="H10" t="n">
-        <v>2</v>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>risotto poulet chorizo</t>
+        </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>gingembre</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr"/>
-      <c r="C11" t="inlineStr"/>
+          <t>parmesan</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>auchan</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>parmesan râpé</t>
+        </is>
+      </c>
       <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
       <c r="G11" t="inlineStr"/>
-      <c r="H11" t="n">
-        <v>2</v>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>risotto poulet chorizo</t>
+        </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>pois chiches en boîte</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr"/>
-      <c r="C12" t="inlineStr"/>
+          <t>oignons</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>leclerc</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>oignons jaunes filet</t>
+        </is>
+      </c>
       <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
       <c r="G12" t="inlineStr"/>
-      <c r="H12" t="n">
-        <v>2</v>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>risotto poulet chorizo</t>
+        </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>poivrons</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr"/>
-      <c r="C13" t="inlineStr"/>
+          <t>lentilles</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>leclerc</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>lentilles vertes origine France</t>
+        </is>
+      </c>
       <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>500</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
       <c r="G13" t="inlineStr"/>
-      <c r="H13" t="n">
-        <v>2</v>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>lentilles lardons</t>
+        </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>tomates concassées</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr"/>
-      <c r="C14" t="inlineStr"/>
+          <t>lentilles</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>carrefour</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>lentilles vertes origine France</t>
+        </is>
+      </c>
       <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr"/>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>500</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
       <c r="G14" t="inlineStr"/>
-      <c r="H14" t="n">
-        <v>2</v>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>lentilles lardons</t>
+        </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>brocolis</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr"/>
-      <c r="C15" t="inlineStr"/>
+          <t>lardons fumés</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>leclerc</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>allumettes de lardons fumés</t>
+        </is>
+      </c>
       <c r="D15" t="inlineStr"/>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr"/>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
       <c r="G15" t="inlineStr"/>
-      <c r="H15" t="n">
-        <v>1</v>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>lentilles lardons</t>
+        </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>bœuf en lanières</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr"/>
-      <c r="C16" t="inlineStr"/>
+          <t>lardons fumés</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>intermarche</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>allumettes de lardons fumés</t>
+        </is>
+      </c>
       <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr"/>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
       <c r="G16" t="inlineStr"/>
-      <c r="H16" t="n">
-        <v>1</v>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>lentilles lardons</t>
+        </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>bœuf haché 5 %</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr"/>
-      <c r="C17" t="inlineStr"/>
+          <t>carottes</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>leclerc</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>carottes sachet</t>
+        </is>
+      </c>
       <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
       <c r="G17" t="inlineStr"/>
-      <c r="H17" t="n">
-        <v>1</v>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>lentilles lardons</t>
+        </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>cabillaud</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr"/>
-      <c r="C18" t="inlineStr"/>
+          <t>ail</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>leclerc</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>ail sachet</t>
+        </is>
+      </c>
       <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr"/>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>pièce</t>
+        </is>
+      </c>
       <c r="G18" t="inlineStr"/>
-      <c r="H18" t="n">
-        <v>1</v>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>lentilles lardons</t>
+        </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>carottes</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr"/>
-      <c r="C19" t="inlineStr"/>
+          <t>bouquet garni</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>carrefour</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>bouquet garni thym laurier</t>
+        </is>
+      </c>
       <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr"/>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>pièce</t>
+        </is>
+      </c>
       <c r="G19" t="inlineStr"/>
-      <c r="H19" t="n">
-        <v>1</v>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>lentilles lardons</t>
+        </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>champignons de Paris</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr"/>
-      <c r="C20" t="inlineStr"/>
+          <t>nouilles ramen</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>joybuy</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>nouilles ramen</t>
+        </is>
+      </c>
       <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>500</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
       <c r="G20" t="inlineStr"/>
-      <c r="H20" t="n">
-        <v>1</v>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>ramen gourmand</t>
+        </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>chou chinois</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr"/>
-      <c r="C21" t="inlineStr"/>
+          <t>nouilles ramen</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>carrefour</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>nouilles ramen</t>
+        </is>
+      </c>
       <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr"/>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>250</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
       <c r="G21" t="inlineStr"/>
-      <c r="H21" t="n">
-        <v>1</v>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>ramen gourmand</t>
+        </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>citrons verts</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr"/>
-      <c r="C22" t="inlineStr"/>
+          <t>pâte miso</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>joybuy</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>miso blanc</t>
+        </is>
+      </c>
       <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr"/>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>300</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
       <c r="G22" t="inlineStr"/>
-      <c r="H22" t="n">
-        <v>1</v>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>ramen gourmand</t>
+        </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>fromage blanc</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr"/>
-      <c r="C23" t="inlineStr"/>
+          <t>mirin</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>joybuy</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>mirin</t>
+        </is>
+      </c>
       <c r="D23" t="inlineStr"/>
-      <c r="E23" t="inlineStr"/>
-      <c r="F23" t="inlineStr"/>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>300</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>ml</t>
+        </is>
+      </c>
       <c r="G23" t="inlineStr"/>
-      <c r="H23" t="n">
-        <v>1</v>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>ramen gourmand</t>
+        </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>fécule de maïs</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr"/>
-      <c r="C24" t="inlineStr"/>
+          <t>sauce soja claire</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>joybuy</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>sauce soja claire</t>
+        </is>
+      </c>
       <c r="D24" t="inlineStr"/>
-      <c r="E24" t="inlineStr"/>
-      <c r="F24" t="inlineStr"/>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>l</t>
+        </is>
+      </c>
       <c r="G24" t="inlineStr"/>
-      <c r="H24" t="n">
-        <v>1</v>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>ramen gourmand</t>
+        </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>graines de sésame</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr"/>
-      <c r="C25" t="inlineStr"/>
+          <t>sauce soja foncée</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>joybuy</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>sauce soja foncée</t>
+        </is>
+      </c>
       <c r="D25" t="inlineStr"/>
-      <c r="E25" t="inlineStr"/>
-      <c r="F25" t="inlineStr"/>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>l</t>
+        </is>
+      </c>
       <c r="G25" t="inlineStr"/>
-      <c r="H25" t="n">
-        <v>1</v>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>ramen gourmand</t>
+        </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>haricots rouges en boîte</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr"/>
-      <c r="C26" t="inlineStr"/>
+          <t>huile de sésame</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>joybuy</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>huile de sésame grillé</t>
+        </is>
+      </c>
       <c r="D26" t="inlineStr"/>
-      <c r="E26" t="inlineStr"/>
-      <c r="F26" t="inlineStr"/>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>250</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>ml</t>
+        </is>
+      </c>
       <c r="G26" t="inlineStr"/>
-      <c r="H26" t="n">
-        <v>1</v>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>ramen gourmand</t>
+        </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>haricots verts</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr"/>
-      <c r="C27" t="inlineStr"/>
+          <t>champignons shiitake</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>joybuy</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>shiitake séchés</t>
+        </is>
+      </c>
       <c r="D27" t="inlineStr"/>
-      <c r="E27" t="inlineStr"/>
-      <c r="F27" t="inlineStr"/>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
       <c r="G27" t="inlineStr"/>
-      <c r="H27" t="n">
-        <v>1</v>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>ramen gourmand</t>
+        </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>lentilles corail</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr"/>
-      <c r="C28" t="inlineStr"/>
+          <t>algues nori</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>joybuy</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>feuilles de nori</t>
+        </is>
+      </c>
       <c r="D28" t="inlineStr"/>
-      <c r="E28" t="inlineStr"/>
-      <c r="F28" t="inlineStr"/>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>pièce</t>
+        </is>
+      </c>
       <c r="G28" t="inlineStr"/>
-      <c r="H28" t="n">
-        <v>1</v>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>ramen gourmand</t>
+        </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>nouilles soba</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr"/>
-      <c r="C29" t="inlineStr"/>
+          <t>gingembre</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>joybuy</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>gingembre frais</t>
+        </is>
+      </c>
       <c r="D29" t="inlineStr"/>
-      <c r="E29" t="inlineStr"/>
-      <c r="F29" t="inlineStr"/>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
       <c r="G29" t="inlineStr"/>
-      <c r="H29" t="n">
-        <v>1</v>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>ramen gourmand</t>
+        </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>pâtes</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr"/>
-      <c r="C30" t="inlineStr"/>
+          <t>poitrine de porc</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>leclerc</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>poitrine de porc fraîche</t>
+        </is>
+      </c>
       <c r="D30" t="inlineStr"/>
-      <c r="E30" t="inlineStr"/>
-      <c r="F30" t="inlineStr"/>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>500</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
       <c r="G30" t="inlineStr"/>
-      <c r="H30" t="n">
-        <v>1</v>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>ramen gourmand</t>
+        </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>saumon</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr"/>
-      <c r="C31" t="inlineStr"/>
+          <t>œufs</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>leclerc</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>œufs label Bleu-Blanc-Cœur</t>
+        </is>
+      </c>
       <c r="D31" t="inlineStr"/>
-      <c r="E31" t="inlineStr"/>
-      <c r="F31" t="inlineStr"/>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>pièce</t>
+        </is>
+      </c>
       <c r="G31" t="inlineStr"/>
-      <c r="H31" t="n">
-        <v>1</v>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>ramen gourmand</t>
+        </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>tomates cerises</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr"/>
-      <c r="C32" t="inlineStr"/>
+          <t>oignons nouveaux</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>carrefour</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>oignons nouveaux botte</t>
+        </is>
+      </c>
       <c r="D32" t="inlineStr"/>
-      <c r="E32" t="inlineStr"/>
-      <c r="F32" t="inlineStr"/>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>pièce</t>
+        </is>
+      </c>
       <c r="G32" t="inlineStr"/>
-      <c r="H32" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>tortillas de blé</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr"/>
-      <c r="C33" t="inlineStr"/>
-      <c r="D33" t="inlineStr"/>
-      <c r="E33" t="inlineStr"/>
-      <c r="F33" t="inlineStr"/>
-      <c r="G33" t="inlineStr"/>
-      <c r="H33" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>épinards</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr"/>
-      <c r="C34" t="inlineStr"/>
-      <c r="D34" t="inlineStr"/>
-      <c r="E34" t="inlineStr"/>
-      <c r="F34" t="inlineStr"/>
-      <c r="G34" t="inlineStr"/>
-      <c r="H34" t="n">
-        <v>1</v>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>ramen gourmand</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -1312,8 +1838,6 @@
           <t>lessive</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr"/>
-      <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
           <t>entretien</t>

</xml_diff>